<commit_message>
Enhance criticality handling in QA loop processing
- Introduced criticality classification and alternatives for evidence candidates in `soroka-run.ts`, improving the handling of conflicts and material uncertainties.
- Updated JSON artifacts to include `criticality` and `alternatives` fields for better data representation.
- Modified the Excel fill process to flag critical items and material uncertainties, ensuring they are visually highlighted in the output.
- Adjusted the results table component to display criticality information, enhancing user awareness of flagged items during review.

This update aims to improve the accuracy and clarity of data processing in the QA loop, facilitating better decision-making based on criticality assessments.
</commit_message>
<xml_diff>
--- a/scripts/qa-loop/artifacts/hm/סקר חוזה - מרלוג HM — AI.xlsx
+++ b/scripts/qa-loop/artifacts/hm/סקר חוזה - מרלוג HM — AI.xlsx
@@ -435,6 +435,58 @@
 </workbook>
 </file>
 
+<file path=xl/comments64.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="D27" authorId="0">
+      <text>
+        <r>
+          <t>⚠ שדה מהותי (כסף/בטיחות) שלא נמצא לו מקור — יש לבדוק ידנית מול מסמכי המכרז.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D36" authorId="0">
+      <text>
+        <r>
+          <t>⚠ שדה מהותי (כסף/בטיחות) שלא נמצא לו מקור — יש לבדוק ידנית מול מסמכי המכרז.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D43" authorId="0">
+      <text>
+        <r>
+          <t>⚠ שדה מהותי (כסף/בטיחות) שלא נמצא לו מקור — יש לבדוק ידנית מול מסמכי המכרז.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D44" authorId="0">
+      <text>
+        <r>
+          <t>⚠ שדה מהותי (כסף/בטיחות) שלא נמצא לו מקור — יש לבדוק ידנית מול מסמכי המכרז.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D51" authorId="0">
+      <text>
+        <r>
+          <t>⚠ שדה מהותי (כסף/בטיחות) שלא נמצא לו מקור — יש לבדוק ידנית מול מסמכי המכרז.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D54" authorId="0">
+      <text>
+        <r>
+          <t>⚠ שדה מהותי (כסף/בטיחות) שלא נמצא לו מקור — יש לבדוק ידנית מול מסמכי המכרז.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="164">
   <si>
@@ -1079,7 +1131,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1104,6 +1156,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="37">
     <border>
@@ -1557,7 +1614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" readingOrder="2"/>
@@ -1611,6 +1668,9 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1692,6 +1752,9 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="49" fontId="8" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -1710,8 +1773,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" readingOrder="2"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -1743,6 +1809,9 @@
     <xf numFmtId="49" fontId="10" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -1760,6 +1829,9 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
@@ -2252,7 +2324,7 @@
       <c r="C8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="20">
         <v>46124</v>
       </c>
       <c r="E8" s="1"/>
@@ -2270,174 +2342,174 @@
     </row>
     <row r="10" ht="30.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="21" t="s">
+      <c r="B10" s="21"/>
+      <c r="C10" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="23" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="1"/>
     </row>
     <row r="11" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="26"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="29"/>
+      <c r="E12" s="30"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="16"/>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="29"/>
+      <c r="E13" s="30"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="16"/>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="30" t="s">
+      <c r="D14" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="E14" s="29"/>
+      <c r="E14" s="30"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="16"/>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="30" t="s">
+      <c r="D15" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="29"/>
+      <c r="E15" s="30"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="30" t="s">
+      <c r="D16" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="29"/>
+      <c r="E16" s="30"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="16"/>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="30" t="s">
+      <c r="D17" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="29"/>
+      <c r="E17" s="30"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="16"/>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="30" t="s">
+      <c r="D18" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="29"/>
+      <c r="E18" s="30"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="16"/>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="30" t="s">
+      <c r="D19" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="29"/>
+      <c r="E19" s="30"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="32" t="s">
+      <c r="B20" s="32"/>
+      <c r="C20" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="33"/>
-      <c r="E20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="35"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="32" t="s">
+      <c r="B21" s="32"/>
+      <c r="C21" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="33" t="s">
+      <c r="D21" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="E21" s="34"/>
+      <c r="E21" s="35"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="32" t="s">
+      <c r="B22" s="32"/>
+      <c r="C22" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="33"/>
-      <c r="E22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="35"/>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="36" t="s">
+      <c r="B23" s="36"/>
+      <c r="C23" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="37"/>
+      <c r="D23" s="38"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
     </row>
     <row r="24" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="39"/>
-      <c r="D24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="41"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="41"/>
-      <c r="C25" s="42" t="s">
+      <c r="B25" s="42"/>
+      <c r="C25" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="44" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="5"/>
@@ -2447,10 +2519,10 @@
     <row r="26" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="44" t="s">
+      <c r="C26" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="D26" s="28" t="s">
+      <c r="D26" s="29" t="s">
         <v>42</v>
       </c>
       <c r="E26" s="5"/>
@@ -2458,33 +2530,33 @@
       <c r="G26" s="5"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B27" s="45"/>
-      <c r="C27" s="44" t="s">
+      <c r="B27" s="46"/>
+      <c r="C27" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="D27" s="28"/>
+      <c r="D27" s="47"/>
       <c r="E27" s="1"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
     </row>
     <row r="28" ht="36.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
-      <c r="B28" s="38" t="s">
+      <c r="B28" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="C28" s="39"/>
-      <c r="D28" s="40"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="41"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
-      <c r="B29" s="45"/>
-      <c r="C29" s="44" t="s">
+      <c r="B29" s="46"/>
+      <c r="C29" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="D29" s="28">
+      <c r="D29" s="29">
         <v>24</v>
       </c>
       <c r="E29" s="1"/>
@@ -2493,11 +2565,11 @@
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
-      <c r="B30" s="45"/>
-      <c r="C30" s="44" t="s">
+      <c r="B30" s="46"/>
+      <c r="C30" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="D30" s="28" t="s">
+      <c r="D30" s="29" t="s">
         <v>47</v>
       </c>
       <c r="E30" s="1"/>
@@ -2506,11 +2578,11 @@
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="46" t="s">
+      <c r="B31" s="36"/>
+      <c r="C31" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="D31" s="47" t="s">
+      <c r="D31" s="49" t="s">
         <v>49</v>
       </c>
       <c r="E31" s="1"/>
@@ -2519,33 +2591,33 @@
     </row>
     <row r="32" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="5"/>
-      <c r="B32" s="35"/>
-      <c r="C32" s="46" t="s">
+      <c r="B32" s="36"/>
+      <c r="C32" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="D32" s="47"/>
+      <c r="D32" s="49"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
     </row>
     <row r="33" ht="36.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
-      <c r="B33" s="38" t="s">
+      <c r="B33" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="39"/>
-      <c r="D33" s="40"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="41"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
     </row>
     <row r="34" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
-      <c r="B34" s="48"/>
-      <c r="C34" s="49" t="s">
+      <c r="B34" s="50"/>
+      <c r="C34" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="D34" s="43">
+      <c r="D34" s="44">
         <v>5000</v>
       </c>
       <c r="E34" s="1"/>
@@ -2554,11 +2626,11 @@
     </row>
     <row r="35" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
-      <c r="B35" s="45"/>
-      <c r="C35" s="44" t="s">
+      <c r="B35" s="46"/>
+      <c r="C35" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="D35" s="28" t="s">
+      <c r="D35" s="29" t="s">
         <v>54</v>
       </c>
       <c r="E35" s="1"/>
@@ -2567,21 +2639,21 @@
     </row>
     <row r="36" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
-      <c r="B36" s="45"/>
-      <c r="C36" s="44" t="s">
+      <c r="B36" s="46"/>
+      <c r="C36" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D36" s="28"/>
+      <c r="D36" s="47"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
     </row>
     <row r="37" ht="36.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B37" s="45"/>
-      <c r="C37" s="50" t="s">
+      <c r="B37" s="46"/>
+      <c r="C37" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="D37" s="28" t="s">
+      <c r="D37" s="29" t="s">
         <v>57</v>
       </c>
       <c r="E37" s="1"/>
@@ -2589,11 +2661,11 @@
       <c r="G37" s="1"/>
     </row>
     <row r="38" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B38" s="45"/>
-      <c r="C38" s="44" t="s">
+      <c r="B38" s="46"/>
+      <c r="C38" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="D38" s="28" t="s">
+      <c r="D38" s="29" t="s">
         <v>59</v>
       </c>
       <c r="E38" s="1"/>
@@ -2601,11 +2673,11 @@
       <c r="G38" s="5"/>
     </row>
     <row r="39" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B39" s="45"/>
-      <c r="C39" s="44" t="s">
+      <c r="B39" s="46"/>
+      <c r="C39" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="D39" s="28" t="s">
+      <c r="D39" s="29" t="s">
         <v>61</v>
       </c>
       <c r="E39" s="1"/>
@@ -2613,11 +2685,11 @@
       <c r="G39" s="5"/>
     </row>
     <row r="40" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B40" s="45"/>
-      <c r="C40" s="44" t="s">
+      <c r="B40" s="46"/>
+      <c r="C40" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="D40" s="28" t="s">
+      <c r="D40" s="29" t="s">
         <v>63</v>
       </c>
       <c r="E40" s="1"/>
@@ -2625,35 +2697,35 @@
       <c r="G40" s="5"/>
     </row>
     <row r="41" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B41" s="45"/>
-      <c r="C41" s="44" t="s">
+      <c r="B41" s="46"/>
+      <c r="C41" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="28" t="s">
+      <c r="D41" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="E41" s="51"/>
+      <c r="E41" s="53"/>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
     </row>
     <row r="42" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B42" s="45"/>
-      <c r="C42" s="44" t="s">
+      <c r="B42" s="46"/>
+      <c r="C42" s="45" t="s">
         <v>66</v>
       </c>
-      <c r="D42" s="28" t="s">
+      <c r="D42" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="E42" s="51"/>
+      <c r="E42" s="53"/>
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
     </row>
     <row r="43" ht="180.6" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="16"/>
-      <c r="C43" s="44" t="s">
+      <c r="C43" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="D43" s="52" t="s">
+      <c r="D43" s="54" t="s">
         <v>69</v>
       </c>
       <c r="E43" s="1"/>
@@ -2662,34 +2734,34 @@
     </row>
     <row r="44" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="16"/>
-      <c r="C44" s="44" t="s">
+      <c r="C44" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="D44" s="30"/>
+      <c r="D44" s="55"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
     </row>
     <row r="45" ht="28.5" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B45" s="45"/>
-      <c r="C45" s="44" t="s">
+      <c r="B45" s="46"/>
+      <c r="C45" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="D45" s="53" t="s">
+      <c r="D45" s="56" t="s">
         <v>72</v>
       </c>
-      <c r="E45" s="54" t="s">
+      <c r="E45" s="57" t="s">
         <v>73</v>
       </c>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
     </row>
     <row r="46" ht="15.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B46" s="45"/>
-      <c r="C46" s="44" t="s">
+      <c r="B46" s="46"/>
+      <c r="C46" s="45" t="s">
         <v>74</v>
       </c>
-      <c r="D46" s="30" t="s">
+      <c r="D46" s="31" t="s">
         <v>75</v>
       </c>
       <c r="E46" s="1"/>
@@ -2697,21 +2769,21 @@
       <c r="G46" s="5"/>
     </row>
     <row r="47" ht="21" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B47" s="55" t="s">
+      <c r="B47" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="C47" s="56"/>
-      <c r="D47" s="57"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="60"/>
       <c r="E47" s="1"/>
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
     </row>
     <row r="48" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B48" s="58"/>
-      <c r="C48" s="59" t="s">
+      <c r="B48" s="61"/>
+      <c r="C48" s="62" t="s">
         <v>77</v>
       </c>
-      <c r="D48" s="60" t="s">
+      <c r="D48" s="63" t="s">
         <v>78</v>
       </c>
       <c r="E48" s="1"/>
@@ -2719,11 +2791,11 @@
       <c r="G48" s="5"/>
     </row>
     <row r="49" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B49" s="45"/>
+      <c r="B49" s="46"/>
       <c r="C49" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D49" s="61" t="s">
+      <c r="D49" s="64" t="s">
         <v>80</v>
       </c>
       <c r="E49" s="1"/>
@@ -2731,59 +2803,59 @@
       <c r="G49" s="5"/>
     </row>
     <row r="50" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B50" s="45"/>
-      <c r="C50" s="62" t="s">
+      <c r="B50" s="46"/>
+      <c r="C50" s="65" t="s">
         <v>81</v>
       </c>
-      <c r="D50" s="61"/>
+      <c r="D50" s="64"/>
       <c r="E50" s="1"/>
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
     </row>
     <row r="51" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B51" s="45"/>
+      <c r="B51" s="46"/>
       <c r="C51" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D51" s="61"/>
+      <c r="D51" s="66"/>
       <c r="E51" s="1"/>
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B52" s="63"/>
-      <c r="C52" s="64"/>
-      <c r="D52" s="65"/>
+      <c r="B52" s="67"/>
+      <c r="C52" s="68"/>
+      <c r="D52" s="69"/>
       <c r="E52" s="1"/>
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
     </row>
     <row r="53" ht="36.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B53" s="66" t="s">
+      <c r="B53" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="C53" s="67"/>
-      <c r="D53" s="68"/>
+      <c r="C53" s="71"/>
+      <c r="D53" s="72"/>
       <c r="E53" s="1"/>
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
     </row>
     <row r="54" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B54" s="41"/>
-      <c r="C54" s="42" t="s">
+      <c r="B54" s="42"/>
+      <c r="C54" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D54" s="43"/>
+      <c r="D54" s="73"/>
       <c r="E54" s="1"/>
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B55" s="69"/>
-      <c r="C55" s="70" t="s">
+      <c r="B55" s="74"/>
+      <c r="C55" s="75" t="s">
         <v>85</v>
       </c>
-      <c r="D55" s="71" t="s">
+      <c r="D55" s="76" t="s">
         <v>86</v>
       </c>
       <c r="E55" s="1"/>
@@ -2791,21 +2863,21 @@
     </row>
     <row r="56" ht="36.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="5"/>
-      <c r="B56" s="38" t="s">
+      <c r="B56" s="39" t="s">
         <v>87</v>
       </c>
-      <c r="C56" s="39"/>
-      <c r="D56" s="40"/>
+      <c r="C56" s="40"/>
+      <c r="D56" s="41"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
     </row>
     <row r="57" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B57" s="72"/>
-      <c r="C57" s="44" t="s">
+      <c r="B57" s="77"/>
+      <c r="C57" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="D57" s="28" t="s">
+      <c r="D57" s="29" t="s">
         <v>89</v>
       </c>
       <c r="E57" s="1"/>
@@ -2813,41 +2885,41 @@
       <c r="G57" s="5"/>
     </row>
     <row r="58" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B58" s="45"/>
-      <c r="C58" s="44" t="s">
+      <c r="B58" s="46"/>
+      <c r="C58" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="D58" s="28" t="s">
+      <c r="D58" s="29" t="s">
         <v>91</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
     </row>
     <row r="59" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B59" s="45"/>
-      <c r="C59" s="44" t="s">
+      <c r="B59" s="46"/>
+      <c r="C59" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="D59" s="28"/>
+      <c r="D59" s="29"/>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
     </row>
     <row r="60" ht="36.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B60" s="72"/>
-      <c r="C60" s="50" t="s">
+      <c r="B60" s="77"/>
+      <c r="C60" s="52" t="s">
         <v>93</v>
       </c>
-      <c r="D60" s="28"/>
+      <c r="D60" s="29"/>
       <c r="E60" s="1"/>
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
     </row>
     <row r="61" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B61" s="72"/>
-      <c r="C61" s="44" t="s">
+      <c r="B61" s="77"/>
+      <c r="C61" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="D61" s="28" t="s">
+      <c r="D61" s="29" t="s">
         <v>95</v>
       </c>
       <c r="E61" s="1"/>
@@ -2856,10 +2928,10 @@
     </row>
     <row r="62" ht="36.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B62" s="16"/>
-      <c r="C62" s="50" t="s">
+      <c r="C62" s="52" t="s">
         <v>96</v>
       </c>
-      <c r="D62" s="28" t="s">
+      <c r="D62" s="29" t="s">
         <v>97</v>
       </c>
       <c r="E62" s="1"/>
@@ -2867,11 +2939,11 @@
       <c r="G62" s="5"/>
     </row>
     <row r="63" ht="15.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B63" s="31"/>
-      <c r="C63" s="73" t="s">
+      <c r="B63" s="32"/>
+      <c r="C63" s="78" t="s">
         <v>98</v>
       </c>
-      <c r="D63" s="28" t="s">
+      <c r="D63" s="29" t="s">
         <v>99</v>
       </c>
       <c r="E63" s="1"/>
@@ -2879,70 +2951,70 @@
       <c r="G63" s="5"/>
     </row>
     <row r="64" ht="36.75" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B64" s="38" t="s">
+      <c r="B64" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="C64" s="39"/>
-      <c r="D64" s="40"/>
+      <c r="C64" s="40"/>
+      <c r="D64" s="41"/>
       <c r="E64" s="1"/>
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
     </row>
     <row r="65" ht="36.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B65" s="48"/>
-      <c r="C65" s="49" t="s">
+      <c r="B65" s="50"/>
+      <c r="C65" s="51" t="s">
         <v>101</v>
       </c>
-      <c r="D65" s="43" t="s">
+      <c r="D65" s="44" t="s">
         <v>102</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="5"/>
     </row>
     <row r="66" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B66" s="74"/>
-      <c r="C66" s="70" t="s">
+      <c r="B66" s="79"/>
+      <c r="C66" s="75" t="s">
         <v>103</v>
       </c>
-      <c r="D66" s="71" t="s">
+      <c r="D66" s="76" t="s">
         <v>104</v>
       </c>
       <c r="E66" s="1"/>
       <c r="F66" s="5"/>
     </row>
     <row r="67" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B67" s="74"/>
-      <c r="C67" s="70" t="s">
+      <c r="B67" s="79"/>
+      <c r="C67" s="75" t="s">
         <v>105</v>
       </c>
-      <c r="D67" s="71" t="s">
+      <c r="D67" s="76" t="s">
         <v>106</v>
       </c>
       <c r="E67" s="1"/>
       <c r="F67" s="5"/>
     </row>
     <row r="68" ht="15.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B68" s="74"/>
-      <c r="C68" s="70"/>
-      <c r="D68" s="71"/>
+      <c r="B68" s="79"/>
+      <c r="C68" s="75"/>
+      <c r="D68" s="76"/>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
     </row>
     <row r="69" ht="36.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B69" s="38" t="s">
+      <c r="B69" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="C69" s="39"/>
-      <c r="D69" s="40"/>
+      <c r="C69" s="40"/>
+      <c r="D69" s="41"/>
       <c r="E69" s="1"/>
       <c r="F69" s="5"/>
     </row>
     <row r="70" ht="15" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B70" s="16"/>
-      <c r="C70" s="50" t="s">
+      <c r="C70" s="52" t="s">
         <v>108</v>
       </c>
-      <c r="D70" s="28" t="s">
+      <c r="D70" s="29" t="s">
         <v>109</v>
       </c>
       <c r="E70" s="1"/>
@@ -2950,110 +3022,110 @@
       <c r="G70" s="5"/>
     </row>
     <row r="71" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B71" s="48"/>
-      <c r="C71" s="42" t="s">
+      <c r="B71" s="50"/>
+      <c r="C71" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="D71" s="75" t="s">
+      <c r="D71" s="80" t="s">
         <v>111</v>
       </c>
       <c r="E71" s="1"/>
       <c r="F71" s="5"/>
     </row>
     <row r="72" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B72" s="45"/>
-      <c r="C72" s="44" t="s">
+      <c r="B72" s="46"/>
+      <c r="C72" s="45" t="s">
         <v>112</v>
       </c>
-      <c r="D72" s="75" t="s">
+      <c r="D72" s="80" t="s">
         <v>113</v>
       </c>
       <c r="E72" s="1"/>
       <c r="F72" s="1"/>
     </row>
     <row r="73" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B73" s="45"/>
-      <c r="C73" s="44" t="s">
+      <c r="B73" s="46"/>
+      <c r="C73" s="45" t="s">
         <v>114</v>
       </c>
-      <c r="D73" s="75" t="s">
+      <c r="D73" s="80" t="s">
         <v>115</v>
       </c>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
     </row>
     <row r="74" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B74" s="45"/>
-      <c r="C74" s="44" t="s">
+      <c r="B74" s="46"/>
+      <c r="C74" s="45" t="s">
         <v>116</v>
       </c>
-      <c r="D74" s="75" t="s">
+      <c r="D74" s="80" t="s">
         <v>117</v>
       </c>
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
     </row>
     <row r="75" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B75" s="45"/>
-      <c r="C75" s="44" t="s">
+      <c r="B75" s="46"/>
+      <c r="C75" s="45" t="s">
         <v>118</v>
       </c>
-      <c r="D75" s="30" t="s">
+      <c r="D75" s="31" t="s">
         <v>119</v>
       </c>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
     </row>
     <row r="76" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B76" s="45"/>
-      <c r="C76" s="44" t="s">
+      <c r="B76" s="46"/>
+      <c r="C76" s="45" t="s">
         <v>120</v>
       </c>
-      <c r="D76" s="30" t="s">
+      <c r="D76" s="31" t="s">
         <v>121</v>
       </c>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
     </row>
     <row r="77" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B77" s="45"/>
-      <c r="C77" s="44" t="s">
+      <c r="B77" s="46"/>
+      <c r="C77" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="D77" s="30" t="s">
+      <c r="D77" s="31" t="s">
         <v>123</v>
       </c>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
     </row>
     <row r="78" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B78" s="45"/>
-      <c r="C78" s="44" t="s">
+      <c r="B78" s="46"/>
+      <c r="C78" s="45" t="s">
         <v>124</v>
       </c>
-      <c r="D78" s="30" t="s">
+      <c r="D78" s="31" t="s">
         <v>125</v>
       </c>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
     </row>
     <row r="79" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B79" s="45"/>
-      <c r="C79" s="50" t="s">
+      <c r="B79" s="46"/>
+      <c r="C79" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="D79" s="28" t="s">
+      <c r="D79" s="29" t="s">
         <v>127</v>
       </c>
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
     </row>
     <row r="80" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B80" s="35"/>
-      <c r="C80" s="46" t="s">
+      <c r="B80" s="36"/>
+      <c r="C80" s="48" t="s">
         <v>128</v>
       </c>
-      <c r="D80" s="47" t="s">
+      <c r="D80" s="49" t="s">
         <v>129</v>
       </c>
       <c r="E80" s="1" t="s">
@@ -3062,165 +3134,165 @@
       <c r="F80" s="1"/>
     </row>
     <row r="81" ht="15.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B81" s="35"/>
-      <c r="C81" s="46" t="s">
+      <c r="B81" s="36"/>
+      <c r="C81" s="48" t="s">
         <v>131</v>
       </c>
-      <c r="D81" s="47" t="s">
+      <c r="D81" s="49" t="s">
         <v>132</v>
       </c>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
     </row>
     <row r="82" ht="21" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B82" s="38" t="s">
+      <c r="B82" s="39" t="s">
         <v>133</v>
       </c>
-      <c r="C82" s="39"/>
-      <c r="D82" s="40"/>
+      <c r="C82" s="40"/>
+      <c r="D82" s="41"/>
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
     </row>
     <row r="83" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B83" s="58"/>
-      <c r="C83" s="59" t="s">
+      <c r="B83" s="61"/>
+      <c r="C83" s="62" t="s">
         <v>134</v>
       </c>
-      <c r="D83" s="76" t="s">
+      <c r="D83" s="81" t="s">
         <v>135</v>
       </c>
-      <c r="E83" s="51"/>
+      <c r="E83" s="53"/>
       <c r="F83" s="1"/>
     </row>
     <row r="84" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B84" s="45"/>
-      <c r="C84" s="77" t="s">
+      <c r="B84" s="46"/>
+      <c r="C84" s="82" t="s">
         <v>136</v>
       </c>
-      <c r="D84" s="75" t="s">
+      <c r="D84" s="80" t="s">
         <v>137</v>
       </c>
-      <c r="E84" s="51"/>
+      <c r="E84" s="53"/>
       <c r="F84" s="1"/>
     </row>
     <row r="85" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B85" s="45"/>
-      <c r="C85" s="77" t="s">
+      <c r="B85" s="46"/>
+      <c r="C85" s="82" t="s">
         <v>138</v>
       </c>
-      <c r="D85" s="75" t="s">
+      <c r="D85" s="80" t="s">
         <v>139</v>
       </c>
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
     </row>
     <row r="86" ht="15.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B86" s="45"/>
+      <c r="B86" s="46"/>
       <c r="C86" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D86" s="75" t="s">
+      <c r="D86" s="80" t="s">
         <v>141</v>
       </c>
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
     </row>
     <row r="87" ht="21" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B87" s="55" t="s">
+      <c r="B87" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="C87" s="56"/>
-      <c r="D87" s="57"/>
-      <c r="E87" s="51"/>
+      <c r="C87" s="59"/>
+      <c r="D87" s="60"/>
+      <c r="E87" s="53"/>
       <c r="F87" s="1"/>
     </row>
     <row r="88" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B88" s="78"/>
-      <c r="C88" s="79" t="s">
+      <c r="B88" s="83"/>
+      <c r="C88" s="84" t="s">
         <v>143</v>
       </c>
-      <c r="D88" s="76"/>
+      <c r="D88" s="81"/>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
     </row>
     <row r="89" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B89" s="16"/>
-      <c r="C89" s="77" t="s">
+      <c r="C89" s="82" t="s">
         <v>144</v>
       </c>
-      <c r="D89" s="75"/>
+      <c r="D89" s="80"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
     </row>
     <row r="90" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B90" s="16"/>
-      <c r="C90" s="77" t="s">
+      <c r="C90" s="82" t="s">
         <v>145</v>
       </c>
-      <c r="D90" s="75"/>
+      <c r="D90" s="80"/>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
     </row>
     <row r="91" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B91" s="80"/>
-      <c r="C91" s="81" t="s">
+      <c r="B91" s="85"/>
+      <c r="C91" s="86" t="s">
         <v>146</v>
       </c>
-      <c r="D91" s="75"/>
+      <c r="D91" s="80"/>
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
     </row>
     <row r="92" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B92" s="80"/>
-      <c r="C92" s="81" t="s">
+      <c r="B92" s="85"/>
+      <c r="C92" s="86" t="s">
         <v>147</v>
       </c>
-      <c r="D92" s="75"/>
+      <c r="D92" s="80"/>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
     </row>
     <row r="93" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B93" s="80"/>
-      <c r="C93" s="81" t="s">
+      <c r="B93" s="85"/>
+      <c r="C93" s="86" t="s">
         <v>148</v>
       </c>
-      <c r="D93" s="75"/>
+      <c r="D93" s="80"/>
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
     </row>
     <row r="94" ht="15.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B94" s="80"/>
-      <c r="C94" s="81"/>
-      <c r="D94" s="75"/>
+      <c r="B94" s="85"/>
+      <c r="C94" s="86"/>
+      <c r="D94" s="80"/>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
     </row>
     <row r="95" ht="21" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B95" s="55" t="s">
+      <c r="B95" s="58" t="s">
         <v>149</v>
       </c>
-      <c r="C95" s="56"/>
-      <c r="D95" s="57"/>
+      <c r="C95" s="59"/>
+      <c r="D95" s="60"/>
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
     </row>
     <row r="96" ht="24.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B96" s="78"/>
-      <c r="C96" s="79" t="s">
+      <c r="B96" s="83"/>
+      <c r="C96" s="84" t="s">
         <v>150</v>
       </c>
-      <c r="D96" s="76" t="s">
+      <c r="D96" s="81" t="s">
         <v>151</v>
       </c>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
     </row>
     <row r="97" ht="24.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B97" s="41"/>
-      <c r="C97" s="82" t="s">
+      <c r="B97" s="42"/>
+      <c r="C97" s="87" t="s">
         <v>152</v>
       </c>
-      <c r="D97" s="83" t="s">
+      <c r="D97" s="88" t="s">
         <v>132</v>
       </c>
       <c r="E97" s="1"/>
@@ -3228,19 +3300,19 @@
     </row>
     <row r="98" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B98" s="16"/>
-      <c r="C98" s="77" t="s">
+      <c r="C98" s="82" t="s">
         <v>153</v>
       </c>
-      <c r="D98" s="75"/>
+      <c r="D98" s="80"/>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
     </row>
     <row r="99" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B99" s="80"/>
-      <c r="C99" s="62" t="s">
+      <c r="B99" s="85"/>
+      <c r="C99" s="65" t="s">
         <v>154</v>
       </c>
-      <c r="D99" s="75"/>
+      <c r="D99" s="80"/>
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
     </row>
@@ -3249,129 +3321,129 @@
       <c r="C100" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="D100" s="75"/>
+      <c r="D100" s="80"/>
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
     </row>
     <row r="101" ht="30" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B101" s="45"/>
-      <c r="C101" s="77" t="s">
+      <c r="B101" s="46"/>
+      <c r="C101" s="82" t="s">
         <v>156</v>
       </c>
-      <c r="D101" s="75"/>
+      <c r="D101" s="80"/>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
     </row>
     <row r="102" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B102" s="84"/>
-      <c r="C102" s="62" t="s">
+      <c r="B102" s="89"/>
+      <c r="C102" s="65" t="s">
         <v>157</v>
       </c>
-      <c r="D102" s="75"/>
+      <c r="D102" s="80"/>
       <c r="E102" s="1"/>
       <c r="F102" s="1"/>
     </row>
     <row r="103" ht="15.75" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B103" s="85"/>
-      <c r="C103" s="86"/>
-      <c r="D103" s="87"/>
+      <c r="B103" s="90"/>
+      <c r="C103" s="91"/>
+      <c r="D103" s="92"/>
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
     </row>
     <row r="104" ht="21" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B104" s="88" t="s">
+      <c r="B104" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="C104" s="89"/>
-      <c r="D104" s="90"/>
+      <c r="C104" s="94"/>
+      <c r="D104" s="95"/>
       <c r="E104" s="1"/>
       <c r="F104" s="1"/>
     </row>
     <row r="105" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B105" s="78"/>
-      <c r="C105" s="91" t="s">
+      <c r="B105" s="83"/>
+      <c r="C105" s="96" t="s">
         <v>158</v>
       </c>
-      <c r="D105" s="76"/>
+      <c r="D105" s="81"/>
       <c r="E105" s="1"/>
       <c r="F105" s="1"/>
     </row>
     <row r="106" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B106" s="16"/>
-      <c r="C106" s="62" t="s">
+      <c r="C106" s="65" t="s">
         <v>159</v>
       </c>
-      <c r="D106" s="75"/>
+      <c r="D106" s="80"/>
       <c r="E106" s="1"/>
       <c r="F106" s="1"/>
     </row>
     <row r="107" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B107" s="80"/>
-      <c r="C107" s="81" t="s">
+      <c r="B107" s="85"/>
+      <c r="C107" s="86" t="s">
         <v>160</v>
       </c>
-      <c r="D107" s="75"/>
+      <c r="D107" s="80"/>
       <c r="E107" s="1"/>
       <c r="F107" s="1"/>
     </row>
     <row r="108" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B108" s="80"/>
-      <c r="C108" s="62"/>
-      <c r="D108" s="75"/>
+      <c r="B108" s="85"/>
+      <c r="C108" s="65"/>
+      <c r="D108" s="80"/>
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
     </row>
     <row r="109" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B109" s="80"/>
-      <c r="C109" s="92"/>
-      <c r="D109" s="93"/>
+      <c r="B109" s="85"/>
+      <c r="C109" s="97"/>
+      <c r="D109" s="98"/>
       <c r="E109" s="1"/>
       <c r="F109" s="1"/>
     </row>
     <row r="110" ht="15" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B110" s="94"/>
-      <c r="C110" s="95"/>
-      <c r="D110" s="96"/>
+      <c r="B110" s="99"/>
+      <c r="C110" s="100"/>
+      <c r="D110" s="101"/>
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
     </row>
     <row r="111" ht="21" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B111" s="66" t="s">
+      <c r="B111" s="70" t="s">
         <v>161</v>
       </c>
-      <c r="C111" s="67"/>
-      <c r="D111" s="68"/>
+      <c r="C111" s="71"/>
+      <c r="D111" s="72"/>
       <c r="E111" s="1"/>
       <c r="F111" s="1"/>
     </row>
     <row r="112" ht="23.45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B112" s="41"/>
-      <c r="C112" s="42" t="s">
+      <c r="B112" s="42"/>
+      <c r="C112" s="43" t="s">
         <v>162</v>
       </c>
-      <c r="D112" s="97" t="s">
+      <c r="D112" s="102" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B113" s="45"/>
-      <c r="C113" s="98"/>
-      <c r="D113" s="75"/>
+      <c r="B113" s="46"/>
+      <c r="C113" s="103"/>
+      <c r="D113" s="80"/>
     </row>
     <row r="114" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B114" s="74"/>
-      <c r="C114" s="92"/>
-      <c r="D114" s="37"/>
+      <c r="B114" s="79"/>
+      <c r="C114" s="97"/>
+      <c r="D114" s="38"/>
     </row>
     <row r="115" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B115" s="69"/>
-      <c r="C115" s="92"/>
-      <c r="D115" s="37"/>
+      <c r="B115" s="74"/>
+      <c r="C115" s="97"/>
+      <c r="D115" s="38"/>
     </row>
     <row r="116" ht="15" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B116" s="85"/>
-      <c r="C116" s="99"/>
-      <c r="D116" s="100"/>
+      <c r="B116" s="90"/>
+      <c r="C116" s="104"/>
+      <c r="D116" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -3396,5 +3468,6 @@
   </mergeCells>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921" bottom="0.7480314960629921" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="83" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>